<commit_message>
Update answer key and final extraction results
</commit_message>
<xml_diff>
--- a/answer_key/answer_key.csv-2.xlsx
+++ b/answer_key/answer_key.csv-2.xlsx
@@ -942,7 +942,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1223,7 +1222,7 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1929</v>
+        <v>996</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -1330,7 +1329,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -1718,7 +1716,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
@@ -2108,7 +2105,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
@@ -2499,7 +2495,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
@@ -2780,7 +2775,7 @@
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>1309</v>
+        <v>734</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>

</xml_diff>